<commit_message>
Codex review and code changes.
</commit_message>
<xml_diff>
--- a/docs/templates/aolf-sheets-template.xlsx
+++ b/docs/templates/aolf-sheets-template.xlsx
@@ -479,7 +479,7 @@
         <v>HP,DSN</v>
       </c>
       <c r="L2" t="str">
-        <v>SSDY</v>
+        <v>Sahaj</v>
       </c>
       <c r="M2" t="str">
         <v>9876543210</v>
@@ -649,7 +649,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -680,7 +680,7 @@
         <v>programs</v>
       </c>
       <c r="B4" t="str">
-        <v>[{"code":"HP","label":"Happiness Program"},{"code":"DSN","label":"Divya Samaj Nirman"},{"code":"SSDY","label":"Sri Sri Dhyana Yoga"}]</v>
+        <v>[{"code":"HP","label":"Happiness Program"},{"code":"VTP","label":"Volunteer Training Program"},{"code":"DSN","label":"Divya Samaj Nirman"},{"code":"IP","label":"Intuition Process"},{"code":"IP2","label":"Intuition Process 2"},{"code":"Sahaj","label":"Sahaj Samadhi Meditation"},{"code":"YES+","label":"YES Plus"}]</v>
       </c>
     </row>
     <row r="5">
@@ -688,7 +688,7 @@
         <v>programDisplayOrder</v>
       </c>
       <c r="B5" t="str">
-        <v>["HP","DSN","SSDY"]</v>
+        <v>["HP","VTP","DSN","IP","IP2","Sahaj","YES+"]</v>
       </c>
     </row>
     <row r="6">
@@ -715,17 +715,9 @@
         <v>91</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>allowedUsers</v>
-      </c>
-      <c r="B9" t="str">
-        <v>volunteer@example.com,admin@example.com</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added course management functionality
</commit_message>
<xml_diff>
--- a/docs/templates/aolf-sheets-template.xlsx
+++ b/docs/templates/aolf-sheets-template.xlsx
@@ -7,7 +7,9 @@
     <sheet name="Members" sheetId="2" r:id="rId2"/>
     <sheet name="Campaigns" sheetId="3" r:id="rId3"/>
     <sheet name="Config" sheetId="4" r:id="rId4"/>
-    <sheet name="AllowedUsers" sheetId="5" r:id="rId5"/>
+    <sheet name="Courses" sheetId="5" r:id="rId5"/>
+    <sheet name="CourseTemplates" sheetId="6" r:id="rId6"/>
+    <sheet name="AllowedUsers" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -724,6 +726,226 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:L2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>courseType</v>
+      </c>
+      <c r="C1" t="str">
+        <v>month</v>
+      </c>
+      <c r="D1" t="str">
+        <v>title</v>
+      </c>
+      <c r="E1" t="str">
+        <v>whatsappTemplate</v>
+      </c>
+      <c r="F1" t="str">
+        <v>pamphletFileId</v>
+      </c>
+      <c r="G1" t="str">
+        <v>pamphletMimeType</v>
+      </c>
+      <c r="H1" t="str">
+        <v>isActive</v>
+      </c>
+      <c r="I1" t="str">
+        <v>createdAt</v>
+      </c>
+      <c r="J1" t="str">
+        <v>updatedAt</v>
+      </c>
+      <c r="K1" t="str">
+        <v>createdBy</v>
+      </c>
+      <c r="L1" t="str">
+        <v>updatedBy</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>crsHpNcr01AbcDefGhiJK</v>
+      </c>
+      <c r="B2" t="str">
+        <v>HP</v>
+      </c>
+      <c r="C2" t="str">
+        <v>2026-08</v>
+      </c>
+      <c r="D2" t="str">
+        <v>HP · August 2026</v>
+      </c>
+      <c r="E2" t="str" xml:space="preserve">
+        <v xml:space="preserve">_*🌿✨HAPPINESS PROGRAM by The Art of Living ✨🌿*_
+😌 Feeling stressed, tired, or overwhelmed?
+Take a pause and discover the power of your breath through Sudarshan Kriya™️ — a life-transforming breathing technique practiced by millions across the globe. 🌍💙
+*Benefits You'll Experience:*
+*Reduces Stress &amp; Anxiety 😌*
+*Improves Sleep Quality 😴✨*
+*Boosts Energy Levels ⚡*
+*Enhances Focus &amp; Mental Clarity 🎯🧠*
+*Strengthens Immunity 💪🛡️*
+*Promotes Emotional Balance 😊🌸*
+*Increases Self-Confidence 🌟*
+*Improves Productivity &amp; Creativity 💡🚀*
+*Relieves Body Aches &amp; Tension 🧘‍♀️💆‍♂️*
+*Brings More Joy, Peace &amp; Happiness 💖🌈*
+📅 Dates: *28 – 30 August*
+🌅 Morning Batch: *6:30 – 9:30 A.M.*
+🌇 Evening Batch: *6:00 – 9:00 P.M.*
+_📍Venue:_
+*Art of Living Nagavara Center*
+*Manyata Tech Park,*
+*Behind Elements Mall*
+*North Bengaluru*
+📞 For Registration &amp; Details: https://aolt.in/874234
+📲 8884560660
+📲 8884561661
+ _🌸 A simple breath. A powerful shift. A happier you. 🌸_
+{courseUrl}</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>true</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-08-01T12:00:00.000Z</v>
+      </c>
+      <c r="J2" t="str">
+        <v>2026-08-01T12:00:00.000Z</v>
+      </c>
+      <c r="K2" t="str">
+        <v>volunteer@example.com</v>
+      </c>
+      <c r="L2" t="str">
+        <v>volunteer@example.com</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:L2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>courseType</v>
+      </c>
+      <c r="B1" t="str">
+        <v>template</v>
+      </c>
+    </row>
+    <row r="2" xml:space="preserve">
+      <c r="A2" t="str">
+        <v>HP</v>
+      </c>
+      <c r="B2" t="str" xml:space="preserve">
+        <v xml:space="preserve">_*🌿✨HAPPINESS PROGRAM by The Art of Living ✨🌿*_
+😌 Feeling stressed, tired, or overwhelmed?
+Take a pause and discover the power of your breath through Sudarshan Kriya™️ — a life-transforming breathing technique practiced by millions across the globe. 🌍💙
+*Benefits You'll Experience:*
+*Reduces Stress &amp; Anxiety 😌*
+*Improves Sleep Quality 😴✨*
+*Boosts Energy Levels ⚡*
+*Enhances Focus &amp; Mental Clarity 🎯🧠*
+*Strengthens Immunity 💪🛡️*
+*Promotes Emotional Balance 😊🌸*
+*Increases Self-Confidence 🌟*
+*Improves Productivity &amp; Creativity 💡🚀*
+*Relieves Body Aches &amp; Tension 🧘‍♀️💆‍♂️*
+*Brings More Joy, Peace &amp; Happiness 💖🌈*
+📅 Dates: *28 – 30 August*
+🌅 Morning Batch: *6:30 – 9:30 A.M.*
+🌇 Evening Batch: *6:00 – 9:00 P.M.*
+_📍Venue:_
+*Art of Living Nagavara Center*
+*Manyata Tech Park,*
+*Behind Elements Mall*
+*North Bengaluru*
+📞 For Registration &amp; Details: https://aolt.in/874234
+📲 8884560660
+📲 8884561661
+ _🌸 A simple breath. A powerful shift. A happier you. 🌸_
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="3" xml:space="preserve">
+      <c r="A3" t="str">
+        <v>VTP</v>
+      </c>
+      <c r="B3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="4" xml:space="preserve">
+      <c r="A4" t="str">
+        <v>DSN</v>
+      </c>
+      <c r="B4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
+      <c r="A5" t="str">
+        <v>IP</v>
+      </c>
+      <c r="B5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="6" xml:space="preserve">
+      <c r="A6" t="str">
+        <v>IP2</v>
+      </c>
+      <c r="B6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>Sahaj</v>
+      </c>
+      <c r="B7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>YES+</v>
+      </c>
+      <c r="B8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Added new feature and code cleaup
</commit_message>
<xml_diff>
--- a/docs/templates/aolf-sheets-template.xlsx
+++ b/docs/templates/aolf-sheets-template.xlsx
@@ -736,7 +736,7 @@
         <v>courseType</v>
       </c>
       <c r="C1" t="str">
-        <v>month</v>
+        <v>programCode</v>
       </c>
       <c r="D1" t="str">
         <v>title</v>
@@ -774,10 +774,10 @@
         <v>HP</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-08</v>
+        <v/>
       </c>
       <c r="D2" t="str">
-        <v>HP · August 2026</v>
+        <v>HP</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
         <v xml:space="preserve">_*🌿✨HAPPINESS PROGRAM by The Art of Living ✨🌿*_
@@ -802,11 +802,12 @@
 *Manyata Tech Park,*
 *Behind Elements Mall*
 *North Bengaluru*
-📞 For Registration &amp; Details: https://aolt.in/874234
+📞 For Registration &amp; Details:
+{courseUrl}
+https://aolt.in/874234
 📲 8884560660
 📲 8884561661
- _🌸 A simple breath. A powerful shift. A happier you. 🌸_
-{courseUrl}</v>
+ _🌸 A simple breath. A powerful shift. A happier you. 🌸_</v>
       </c>
       <c r="F2" t="str">
         <v/>
@@ -839,7 +840,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -876,11 +877,12 @@
 *Manyata Tech Park,*
 *Behind Elements Mall*
 *North Bengaluru*
-📞 For Registration &amp; Details: https://aolt.in/874234
+📞 For Registration &amp; Details:
+{courseUrl}
+https://aolt.in/874234
 📲 8884560660
 📲 8884561661
- _🌸 A simple breath. A powerful shift. A happier you. 🌸_
-{courseUrl}</v>
+ _🌸 A simple breath. A powerful shift. A happier you. 🌸_</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -903,7 +905,7 @@
     </row>
     <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>IP</v>
+        <v>IP-j</v>
       </c>
       <c r="B5" t="str" xml:space="preserve">
         <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
@@ -912,7 +914,7 @@
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>IP2</v>
+        <v>IP-s</v>
       </c>
       <c r="B6" t="str" xml:space="preserve">
         <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
@@ -921,7 +923,7 @@
     </row>
     <row r="7" xml:space="preserve">
       <c r="A7" t="str">
-        <v>Sahaj</v>
+        <v>IP2</v>
       </c>
       <c r="B7" t="str" xml:space="preserve">
         <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
@@ -930,16 +932,25 @@
     </row>
     <row r="8" xml:space="preserve">
       <c r="A8" t="str">
-        <v>YES+</v>
+        <v>Sahaj</v>
       </c>
       <c r="B8" t="str" xml:space="preserve">
         <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
 {courseUrl}</v>
       </c>
     </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>YES+</v>
+      </c>
+      <c r="B9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Hi {name}, you are invited to {course} ({dates}).
+{courseUrl}</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Added short url functionality to the sheets service. This allows for generating short URLs for specific sheets, making it easier to share and access them. The implementation includes a new endpoint in the API that handles the creation of short URLs and redirects users to the original sheet when accessed.
</commit_message>
<xml_diff>
--- a/docs/templates/aolf-sheets-template.xlsx
+++ b/docs/templates/aolf-sheets-template.xlsx
@@ -9,7 +9,8 @@
     <sheet name="Config" sheetId="4" r:id="rId4"/>
     <sheet name="Activities" sheetId="5" r:id="rId5"/>
     <sheet name="CourseTemplates" sheetId="6" r:id="rId6"/>
-    <sheet name="AllowedUsers" sheetId="7" r:id="rId7"/>
+    <sheet name="ShortUrls" sheetId="7" r:id="rId7"/>
+    <sheet name="AllowedUsers" sheetId="8" r:id="rId8"/>
   </sheets>
 </workbook>
 </file>
@@ -1008,6 +1009,50 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>slug</v>
+      </c>
+      <c r="B1" t="str">
+        <v>destinationUrl</v>
+      </c>
+      <c r="C1" t="str">
+        <v>isActive</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>sample</v>
+      </c>
+      <c r="B2" t="str">
+        <v>https://www.artofliving.org/in-en</v>
+      </c>
+      <c r="C2" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>tu/rp</v>
+      </c>
+      <c r="B3" t="str">
+        <v>https://www.artofliving.org/in-en/programs</v>
+      </c>
+      <c r="C3" t="str">
+        <v>true</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C3"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
         <v>email</v>
       </c>
       <c r="B1" t="str">

</xml_diff>